<commit_message>
Personal ID plan: align status convention with the Tasking plan
Match how the Tasking_Workflow_Automation_Test_Plan marks coverage:
- Status column left blank in the case sheet (reserved for manual pass/fail runs).
- Automation Target is the coverage indicator: the test / Maestro flow that covers
  the case, or "Manual only" for the deferred cases (PID_50/60/61/62).
- Legend refreshed to describe the Automation Target convention.

No scope change - PID_48-59 remain automated (verified), PID_50/60/61/62 manual.

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Personal_ID_Automation_Test_Plan.xlsx
+++ b/Personal_ID_Automation_Test_Plan.xlsx
@@ -103,7 +103,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="11">
+  <cellXfs count="13">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
@@ -127,6 +127,10 @@
     <xf numFmtId="0" fontId="0" fillId="6" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="7" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="5" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -771,7 +775,7 @@
     <row r="2">
       <c r="A2" s="4" t="inlineStr">
         <is>
-          <t>Traditional App Install &amp; Login  -  PID_48 through PID_62 (15 cases; 3 web automated, 5 mobile to do, 1 web built/blocked, 4 deferred-manual)</t>
+          <t>Traditional App Install &amp; Login  -  PID_48 to PID_62 (15 cases)</t>
         </is>
       </c>
     </row>
@@ -811,11 +815,7 @@
           <t>Mobile (Maestro) - maestro_mobile/flows/pid_48_link_prompt.yaml</t>
         </is>
       </c>
-      <c r="G3" s="5" t="inlineStr">
-        <is>
-          <t>Done</t>
-        </is>
-      </c>
+      <c r="G3" s="2" t="n"/>
       <c r="H3" s="3" t="inlineStr">
         <is>
           <t>Link-to-PID popup appears after worker password login. VERIFIED on emulator.</t>
@@ -856,11 +856,7 @@
           <t>Mobile (Maestro) - maestro_mobile/flows/pid_49_link_declined.yaml</t>
         </is>
       </c>
-      <c r="G4" s="5" t="inlineStr">
-        <is>
-          <t>Done</t>
-        </is>
-      </c>
+      <c r="G4" s="2" t="n"/>
       <c r="H4" s="3" t="inlineStr">
         <is>
           <t>Select No -&gt; logs into app normally. VERIFIED.</t>
@@ -891,14 +887,10 @@
       </c>
       <c r="F5" s="3" t="inlineStr">
         <is>
-          <t>Manual</t>
-        </is>
-      </c>
-      <c r="G5" s="6" t="inlineStr">
-        <is>
-          <t>Deferred</t>
-        </is>
-      </c>
+          <t>Manual only</t>
+        </is>
+      </c>
+      <c r="G5" s="2" t="n"/>
       <c r="H5" s="3" t="inlineStr">
         <is>
           <t>30-day re-prompt is time-dependent (evaluateLinkOffer offer-date logic); cannot reliably automate in a single session.</t>
@@ -937,11 +929,7 @@
           <t>Mobile (Maestro) - maestro_mobile/flows/pid_51_link_accepted.yaml</t>
         </is>
       </c>
-      <c r="G6" s="5" t="inlineStr">
-        <is>
-          <t>Done</t>
-        </is>
-      </c>
+      <c r="G6" s="2" t="n"/>
       <c r="H6" s="3" t="inlineStr">
         <is>
           <t>Select Yes -&gt; MW linked to PersonalId. VERIFIED.</t>
@@ -980,11 +968,7 @@
           <t>Mobile (Maestro) - maestro_mobile/flows/pid_53_unlink_prompt.yaml</t>
         </is>
       </c>
-      <c r="G7" s="5" t="inlineStr">
-        <is>
-          <t>Done</t>
-        </is>
-      </c>
+      <c r="G7" s="2" t="n"/>
       <c r="H7" s="3" t="inlineStr">
         <is>
           <t>Password login while linked works (covered by the unlink-prompt journey). VERIFIED.</t>
@@ -1025,11 +1009,7 @@
           <t>Mobile (Maestro) - maestro_mobile/flows/pid_53_unlink_prompt.yaml</t>
         </is>
       </c>
-      <c r="G8" s="5" t="inlineStr">
-        <is>
-          <t>Done</t>
-        </is>
-      </c>
+      <c r="G8" s="2" t="n"/>
       <c r="H8" s="3" t="inlineStr">
         <is>
           <t>Unlink-PID popup appears on password login when linked. VERIFIED.</t>
@@ -1070,11 +1050,7 @@
           <t>Mobile (Maestro) - maestro_mobile/flows/pid_54_unlink_accepted.yaml</t>
         </is>
       </c>
-      <c r="G9" s="5" t="inlineStr">
-        <is>
-          <t>Done</t>
-        </is>
-      </c>
+      <c r="G9" s="2" t="n"/>
       <c r="H9" s="3" t="inlineStr">
         <is>
           <t>Yes on unlink popup -&gt; MW unlinked. VERIFIED.</t>
@@ -1114,11 +1090,7 @@
           <t>Mobile (Maestro) - maestro_mobile/flows/pid_55_unlink_declined.yaml</t>
         </is>
       </c>
-      <c r="G10" s="5" t="inlineStr">
-        <is>
-          <t>Done</t>
-        </is>
-      </c>
+      <c r="G10" s="2" t="n"/>
       <c r="H10" s="3" t="inlineStr">
         <is>
           <t>No on unlink popup -&gt; stays linked. VERIFIED.</t>
@@ -1161,11 +1133,7 @@
           <t>Web (Playwright) - tests/test_pid_56_57_58_59.py :: test_pid_56_57_58_personalid_unlink_on_mobile_workers</t>
         </is>
       </c>
-      <c r="G11" s="5" t="inlineStr">
-        <is>
-          <t>Done</t>
-        </is>
-      </c>
+      <c r="G11" s="2" t="n"/>
       <c r="H11" s="3" t="inlineStr">
         <is>
           <t>PersonalID Status column present + valid values. PASS on staging.</t>
@@ -1204,11 +1172,7 @@
           <t>Web (Playwright) - tests/test_pid_56_57_58_59.py :: test_pid_56_57_58_personalid_unlink_on_mobile_workers</t>
         </is>
       </c>
-      <c r="G12" s="5" t="inlineStr">
-        <is>
-          <t>Done</t>
-        </is>
-      </c>
+      <c r="G12" s="2" t="n"/>
       <c r="H12" s="3" t="inlineStr">
         <is>
           <t>Unlink PersonalID action present for linked worker. PASS on staging.</t>
@@ -1244,11 +1208,7 @@
           <t>Web (Playwright) - tests/test_pid_56_57_58_59.py :: test_pid_56_57_58_personalid_unlink_on_mobile_workers</t>
         </is>
       </c>
-      <c r="G13" s="5" t="inlineStr">
-        <is>
-          <t>Done</t>
-        </is>
-      </c>
+      <c r="G13" s="2" t="n"/>
       <c r="H13" s="3" t="inlineStr">
         <is>
           <t>Unlink confirm modal (Cancel/Unlink) -&gt; Cancel (non-destructive). PASS on staging.</t>
@@ -1284,11 +1244,7 @@
           <t>Web (Playwright) - tests/test_pid_56_57_58_59.py :: test_pid_59_confirm_unlink_flips_status (guarded: RUN_DESTRUCTIVE_PID + PID_UNLINK_WORKER)</t>
         </is>
       </c>
-      <c r="G14" s="5" t="inlineStr">
-        <is>
-          <t>Done</t>
-        </is>
-      </c>
+      <c r="G14" s="2" t="n"/>
       <c r="H14" s="3" t="inlineStr">
         <is>
           <t>Unlink flips status to Not Linked/Inactive, then RE-LINKS to restore (HQ 'Link PersonalID' needs no input) so it is idempotent and runs every time. Targets PID_UNLINK_WORKER (default CCC-Automationuser1), falling back to any linked worker; only skips if the domain has no linked worker at all. VERIFIED.</t>
@@ -1319,14 +1275,10 @@
       </c>
       <c r="F15" s="3" t="inlineStr">
         <is>
-          <t>Manual</t>
-        </is>
-      </c>
-      <c r="G15" s="6" t="inlineStr">
-        <is>
-          <t>Deferred</t>
-        </is>
-      </c>
+          <t>Manual only</t>
+        </is>
+      </c>
+      <c r="G15" s="2" t="n"/>
       <c r="H15" s="3" t="inlineStr">
         <is>
           <t>Go to Connect Menu shown for Beta but not Mainline -&gt; needs two APK variants.</t>
@@ -1362,14 +1314,10 @@
       </c>
       <c r="F16" s="3" t="inlineStr">
         <is>
-          <t>Manual</t>
-        </is>
-      </c>
-      <c r="G16" s="6" t="inlineStr">
-        <is>
-          <t>Deferred</t>
-        </is>
-      </c>
+          <t>Manual only</t>
+        </is>
+      </c>
+      <c r="G16" s="2" t="n"/>
       <c r="H16" s="3" t="inlineStr">
         <is>
           <t>Device-1 logout push on Device-2 login -&gt; needs two concurrent devices.</t>
@@ -1396,14 +1344,10 @@
       </c>
       <c r="F17" s="3" t="inlineStr">
         <is>
-          <t>Manual</t>
-        </is>
-      </c>
-      <c r="G17" s="6" t="inlineStr">
-        <is>
-          <t>Deferred</t>
-        </is>
-      </c>
+          <t>Manual only</t>
+        </is>
+      </c>
+      <c r="G17" s="2" t="n"/>
       <c r="H17" s="3" t="inlineStr">
         <is>
           <t>Sign-up gated to Android &gt;= 9 -&gt; needs a device-version matrix.</t>
@@ -1427,67 +1371,67 @@
   <dimension ref="A1:B5"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="18" customWidth="1" min="1" max="1"/>
-    <col width="80" customWidth="1" min="2" max="2"/>
+    <col width="22" customWidth="1" min="1" max="1"/>
+    <col width="92" customWidth="1" min="2" max="2"/>
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="1" t="inlineStr">
+      <c r="A1" s="11" t="inlineStr">
+        <is>
+          <t>Column</t>
+        </is>
+      </c>
+      <c r="B1" s="11" t="inlineStr">
+        <is>
+          <t>Meaning</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>Automation Target</t>
+        </is>
+      </c>
+      <c r="B2" s="12" t="inlineStr">
+        <is>
+          <t>The test / Maestro flow that covers the case (= automated), or 'Manual only' when it is not automated.</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>Phase</t>
+        </is>
+      </c>
+      <c r="B3" s="12" t="inlineStr">
+        <is>
+          <t>1 - Web (Playwright), 2 - Mobile (Maestro), or Manual / Deferred.</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
         <is>
           <t>Status</t>
         </is>
       </c>
-      <c r="B1" s="1" t="inlineStr">
-        <is>
-          <t>Meaning</t>
-        </is>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" s="7" t="inlineStr">
-        <is>
-          <t>Done</t>
-        </is>
-      </c>
-      <c r="B2" s="3" t="inlineStr">
-        <is>
-          <t>Automated and passing on staging.</t>
-        </is>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" s="8" t="inlineStr">
-        <is>
-          <t>To do</t>
-        </is>
-      </c>
-      <c r="B3" s="3" t="inlineStr">
-        <is>
-          <t>In scope; automation not yet written (mobile Maestro phase).</t>
-        </is>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" s="9" t="inlineStr">
-        <is>
-          <t>Built - blocked</t>
-        </is>
-      </c>
-      <c r="B4" s="3" t="inlineStr">
-        <is>
-          <t>Test written but cannot run live until a prerequisite exists (e.g. a linked dedicated worker).</t>
+      <c r="B4" s="12" t="inlineStr">
+        <is>
+          <t>Left blank - reserved for manual pass/fail runs (matches the Tasking plan).</t>
         </is>
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="10" t="inlineStr">
-        <is>
-          <t>Deferred</t>
-        </is>
-      </c>
-      <c r="B5" s="3" t="inlineStr">
-        <is>
-          <t>Not automatable in a single session; tracked as manual (device matrix, 2 devices, timing, build variants).</t>
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>Comments / Notes</t>
+        </is>
+      </c>
+      <c r="B5" s="12" t="inlineStr">
+        <is>
+          <t>Verification notes and behaviour caveats.</t>
         </is>
       </c>
     </row>

</xml_diff>